<commit_message>
deploy: 2026-07-07 05:16 (build 20260707051612)
</commit_message>
<xml_diff>
--- a/cloudflare-deploy/public/library/admin/admin-en.xlsx
+++ b/cloudflare-deploy/public/library/admin/admin-en.xlsx
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1835,6 +1835,114 @@
       <c r="E24" s="15" t="inlineStr">
         <is>
           <t>Listen slowly and repeat clearly to nail the four tones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>📢</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Notice Studio (Poster + Popup)</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Go to the admin menu Notification Center → 📢 Notice Studio. → In the ①Create tab, design a poster with text, images, and video (resize · save on server · reuse). → Press ‘📢 Publish as popup’ on the finished poster to auto-switch to the ②Publish·Popup tab. → In the publish tab, set the display period / stop and publish it as a student-app popup.</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>Promoting an event takes just one flow: ‘Create → Publish as popup’ right away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>🤖</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Command the AI Operations Assistant</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Type a command in the top search bar or speak with the 🎤 mic. → e.g. “Take me to teacher Kim Minji's schedule” → auto-finds that teacher in the weekly schedule and opens it. → e.g. “Open auto-scheduling,” “Go to settlement” to navigate menus. → Press ‘Go now →’ on the AI response card to move to that screen.</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>When you can't recall a menu name, just say what you want to do — it finds its way there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>📔</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Student Voice-Diary Monitor</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Open the 📔 Voice Diary (monitor) card in the admin menu. → Enter the student UID, pick the month to look up, and press ‘Search’. → Open an entry from the list to see the transcript · correction · encouragement · score.</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>‘Nothing shows up’ usually just means that student hasn't left a diary yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>🤖</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Teacher AI-Coaching Review (Ops)</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Go to admin 🧲 Retention Center → 💼 Teacher Coaching tab. → In the ‘🤖 Per-class AI coaching (recent)’ section, review each teacher's latest coaching. → Use each card's quality score · talk ratio · improvement point to plan coaching and training.</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>For teachers whose quality score stays low, coach them together with the teacher training manual.</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F229"/>
+  <dimension ref="A1:F276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4382,44 +4490,583 @@
       <c r="E229" s="33" t="n"/>
       <c r="F229" s="33" t="n"/>
     </row>
+    <row r="231" ht="26" customHeight="1">
+      <c r="A231" s="21" t="inlineStr">
+        <is>
+          <t>22  📢 Notice Studio (Poster + Popup)  —  Design notice/event posters and push them as app popups</t>
+        </is>
+      </c>
+      <c r="B231" s="22" t="n"/>
+      <c r="C231" s="22" t="n"/>
+      <c r="D231" s="22" t="n"/>
+      <c r="E231" s="22" t="n"/>
+      <c r="F231" s="22" t="n"/>
+    </row>
+    <row r="232" ht="42" customHeight="1">
+      <c r="A232" s="23" t="inlineStr">
+        <is>
+          <t>📖 This merges the old ‘Poster Maker’ and ‘Popup Notice’ tools into one place. In the ①Create tab you design a notice/event poster, then hand it straight to the ②Publish·Popup tab to show it as a popup in your academy's student app.</t>
+        </is>
+      </c>
+      <c r="B232" s="24" t="n"/>
+      <c r="C232" s="24" t="n"/>
+      <c r="D232" s="24" t="n"/>
+      <c r="E232" s="24" t="n"/>
+      <c r="F232" s="24" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B233" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="30" customHeight="1">
+      <c r="A234" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B234" s="28" t="inlineStr">
+        <is>
+          <t>Go to the admin menu Notification Center → 📢 Notice Studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="30" customHeight="1">
+      <c r="A235" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B235" s="28" t="inlineStr">
+        <is>
+          <t>In the ①Create tab, design a poster with text, images, and video (resize · save on server · reuse).</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="30" customHeight="1">
+      <c r="A236" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B236" s="28" t="inlineStr">
+        <is>
+          <t>Press ‘📢 Publish as popup’ on the finished poster to auto-switch to the ②Publish·Popup tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="30" customHeight="1">
+      <c r="A237" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B237" s="28" t="inlineStr">
+        <is>
+          <t>In the publish tab, set the display period / stop and publish it as a student-app popup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="24" customHeight="1">
+      <c r="A238" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B238" s="30" t="inlineStr">
+        <is>
+          <t>Poster creation and popup publishing flow through one screen, two tabs — no more confusion.</t>
+        </is>
+      </c>
+      <c r="C238" s="31" t="n"/>
+      <c r="D238" s="31" t="n"/>
+      <c r="E238" s="31" t="n"/>
+      <c r="F238" s="31" t="n"/>
+    </row>
+    <row r="239" ht="24" customHeight="1">
+      <c r="A239" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B239" s="30" t="inlineStr">
+        <is>
+          <t>Posters you make can be saved and reused.</t>
+        </is>
+      </c>
+      <c r="C239" s="31" t="n"/>
+      <c r="D239" s="31" t="n"/>
+      <c r="E239" s="31" t="n"/>
+      <c r="F239" s="31" t="n"/>
+    </row>
+    <row r="240" ht="24" customHeight="1">
+      <c r="A240" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B240" s="30" t="inlineStr">
+        <is>
+          <t>Whichever route you enter from — AI assistant or sidebar search — the correct tab opens.</t>
+        </is>
+      </c>
+      <c r="C240" s="31" t="n"/>
+      <c r="D240" s="31" t="n"/>
+      <c r="E240" s="31" t="n"/>
+      <c r="F240" s="31" t="n"/>
+    </row>
+    <row r="241" ht="26" customHeight="1">
+      <c r="A241" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ Good to know · Existing posters/popups are preserved (it was only merged, nothing was deleted).</t>
+        </is>
+      </c>
+      <c r="B241" s="35" t="n"/>
+      <c r="C241" s="35" t="n"/>
+      <c r="D241" s="35" t="n"/>
+      <c r="E241" s="35" t="n"/>
+      <c r="F241" s="35" t="n"/>
+    </row>
+    <row r="242" ht="30" customHeight="1">
+      <c r="A242" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · Promoting an event takes just one flow: ‘Create → Publish as popup’ right away.</t>
+        </is>
+      </c>
+      <c r="B242" s="33" t="n"/>
+      <c r="C242" s="33" t="n"/>
+      <c r="D242" s="33" t="n"/>
+      <c r="E242" s="33" t="n"/>
+      <c r="F242" s="33" t="n"/>
+    </row>
+    <row r="244" ht="26" customHeight="1">
+      <c r="A244" s="21" t="inlineStr">
+        <is>
+          <t>23  🤖 Command the AI Operations Assistant  —  Navigate with one phrase: “Take me to ○○”</t>
+        </is>
+      </c>
+      <c r="B244" s="22" t="n"/>
+      <c r="C244" s="22" t="n"/>
+      <c r="D244" s="22" t="n"/>
+      <c r="E244" s="22" t="n"/>
+      <c r="F244" s="22" t="n"/>
+    </row>
+    <row r="245" ht="42" customHeight="1">
+      <c r="A245" s="23" t="inlineStr">
+        <is>
+          <t>📖 Type what you want to do into the top search bar (or the bottom-right AI assistant) in plain language, and the AI understands and jumps straight to that screen. It now reliably follows navigation commands like ‘Take me to teacher ○○'s schedule’ or ‘Open auto-scheduling’.</t>
+        </is>
+      </c>
+      <c r="B245" s="24" t="n"/>
+      <c r="C245" s="24" t="n"/>
+      <c r="D245" s="24" t="n"/>
+      <c r="E245" s="24" t="n"/>
+      <c r="F245" s="24" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B246" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="30" customHeight="1">
+      <c r="A247" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B247" s="28" t="inlineStr">
+        <is>
+          <t>Type a command in the top search bar or speak with the 🎤 mic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="30" customHeight="1">
+      <c r="A248" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B248" s="28" t="inlineStr">
+        <is>
+          <t>e.g. “Take me to teacher Kim Minji's schedule” → auto-finds that teacher in the weekly schedule and opens it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="30" customHeight="1">
+      <c r="A249" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B249" s="28" t="inlineStr">
+        <is>
+          <t>e.g. “Open auto-scheduling,” “Go to settlement” to navigate menus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="30" customHeight="1">
+      <c r="A250" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B250" s="28" t="inlineStr">
+        <is>
+          <t>Press ‘Go now →’ on the AI response card to move to that screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="24" customHeight="1">
+      <c r="A251" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B251" s="30" t="inlineStr">
+        <is>
+          <t>Navigation commands actually navigate — far fewer ‘explain only, do nothing’ replies.</t>
+        </is>
+      </c>
+      <c r="C251" s="31" t="n"/>
+      <c r="D251" s="31" t="n"/>
+      <c r="E251" s="31" t="n"/>
+      <c r="F251" s="31" t="n"/>
+    </row>
+    <row r="252" ht="24" customHeight="1">
+      <c r="A252" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B252" s="30" t="inlineStr">
+        <is>
+          <t>Searching a schedule by teacher name auto-fills the search box + filters + scrolls.</t>
+        </is>
+      </c>
+      <c r="C252" s="31" t="n"/>
+      <c r="D252" s="31" t="n"/>
+      <c r="E252" s="31" t="n"/>
+      <c r="F252" s="31" t="n"/>
+    </row>
+    <row r="253" ht="24" customHeight="1">
+      <c r="A253" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B253" s="30" t="inlineStr">
+        <is>
+          <t>For data/statistics questions it also helps with card-style answers.</t>
+        </is>
+      </c>
+      <c r="C253" s="31" t="n"/>
+      <c r="D253" s="31" t="n"/>
+      <c r="E253" s="31" t="n"/>
+      <c r="F253" s="31" t="n"/>
+    </row>
+    <row r="254" ht="26" customHeight="1">
+      <c r="A254" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ Good to know · Commands that actually change things — ‘register · send · modify’ — ask for one more confirmation (a safety guard).</t>
+        </is>
+      </c>
+      <c r="B254" s="35" t="n"/>
+      <c r="C254" s="35" t="n"/>
+      <c r="D254" s="35" t="n"/>
+      <c r="E254" s="35" t="n"/>
+      <c r="F254" s="35" t="n"/>
+    </row>
+    <row r="255" ht="30" customHeight="1">
+      <c r="A255" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · When you can't recall a menu name, just say what you want to do — it finds its way there.</t>
+        </is>
+      </c>
+      <c r="B255" s="33" t="n"/>
+      <c r="C255" s="33" t="n"/>
+      <c r="D255" s="33" t="n"/>
+      <c r="E255" s="33" t="n"/>
+      <c r="F255" s="33" t="n"/>
+    </row>
+    <row r="257" ht="26" customHeight="1">
+      <c r="A257" s="21" t="inlineStr">
+        <is>
+          <t>24  📔 Student Voice-Diary Monitor  —  View each student's English diary · AI correction · score</t>
+        </is>
+      </c>
+      <c r="B257" s="22" t="n"/>
+      <c r="C257" s="22" t="n"/>
+      <c r="D257" s="22" t="n"/>
+      <c r="E257" s="22" t="n"/>
+      <c r="F257" s="22" t="n"/>
+    </row>
+    <row r="258" ht="42" customHeight="1">
+      <c r="A258" s="23" t="inlineStr">
+        <is>
+          <t>📖 View the AI voice diaries students leave, right from the admin screen. Per student, check the transcript · AI correction · encouragement · score by month to encourage consistent writers and gauge their learning.</t>
+        </is>
+      </c>
+      <c r="B258" s="24" t="n"/>
+      <c r="C258" s="24" t="n"/>
+      <c r="D258" s="24" t="n"/>
+      <c r="E258" s="24" t="n"/>
+      <c r="F258" s="24" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B259" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="30" customHeight="1">
+      <c r="A260" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B260" s="28" t="inlineStr">
+        <is>
+          <t>Open the 📔 Voice Diary (monitor) card in the admin menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="30" customHeight="1">
+      <c r="A261" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B261" s="28" t="inlineStr">
+        <is>
+          <t>Enter the student UID, pick the month to look up, and press ‘Search’.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="30" customHeight="1">
+      <c r="A262" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B262" s="28" t="inlineStr">
+        <is>
+          <t>Open an entry from the list to see the transcript · correction · encouragement · score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="24" customHeight="1">
+      <c r="A263" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B263" s="30" t="inlineStr">
+        <is>
+          <t>It only shows up once a student actually writes a diary (the entry point is the 📔 card on the student home).</t>
+        </is>
+      </c>
+      <c r="C263" s="31" t="n"/>
+      <c r="D263" s="31" t="n"/>
+      <c r="E263" s="31" t="n"/>
+      <c r="F263" s="31" t="n"/>
+    </row>
+    <row r="264" ht="24" customHeight="1">
+      <c r="A264" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B264" s="30" t="inlineStr">
+        <is>
+          <t>Find consistent writers and connect them to praise/rewards to lock in the habit.</t>
+        </is>
+      </c>
+      <c r="C264" s="31" t="n"/>
+      <c r="D264" s="31" t="n"/>
+      <c r="E264" s="31" t="n"/>
+      <c r="F264" s="31" t="n"/>
+    </row>
+    <row r="265" ht="30" customHeight="1">
+      <c r="A265" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · ‘Nothing shows up’ usually just means that student hasn't left a diary yet.</t>
+        </is>
+      </c>
+      <c r="B265" s="33" t="n"/>
+      <c r="C265" s="33" t="n"/>
+      <c r="D265" s="33" t="n"/>
+      <c r="E265" s="33" t="n"/>
+      <c r="F265" s="33" t="n"/>
+    </row>
+    <row r="267" ht="26" customHeight="1">
+      <c r="A267" s="21" t="inlineStr">
+        <is>
+          <t>25  🤖 Teacher AI-Coaching Review (Ops)  —  Collected per-class AI coaching · quality scores</t>
+        </is>
+      </c>
+      <c r="B267" s="22" t="n"/>
+      <c r="C267" s="22" t="n"/>
+      <c r="D267" s="22" t="n"/>
+      <c r="E267" s="22" t="n"/>
+      <c r="F267" s="22" t="n"/>
+    </row>
+    <row r="268" ht="42" customHeight="1">
+      <c r="A268" s="23" t="inlineStr">
+        <is>
+          <t>📖 After every class, the AI leaves the teacher a coaching card (strengths · areas to improve · a class-quality score). From the admin screen you can see these gathered by most-recent. Use it as a growth-support / coaching-quality tool — not surveillance.</t>
+        </is>
+      </c>
+      <c r="B268" s="24" t="n"/>
+      <c r="C268" s="24" t="n"/>
+      <c r="D268" s="24" t="n"/>
+      <c r="E268" s="24" t="n"/>
+      <c r="F268" s="24" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B269" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="30" customHeight="1">
+      <c r="A270" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B270" s="28" t="inlineStr">
+        <is>
+          <t>Go to admin 🧲 Retention Center → 💼 Teacher Coaching tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="30" customHeight="1">
+      <c r="A271" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B271" s="28" t="inlineStr">
+        <is>
+          <t>In the ‘🤖 Per-class AI coaching (recent)’ section, review each teacher's latest coaching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="30" customHeight="1">
+      <c r="A272" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B272" s="28" t="inlineStr">
+        <is>
+          <t>Use each card's quality score · talk ratio · improvement point to plan coaching and training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="24" customHeight="1">
+      <c r="A273" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B273" s="30" t="inlineStr">
+        <is>
+          <t>See every teacher's recent coaching at a glance.</t>
+        </is>
+      </c>
+      <c r="C273" s="31" t="n"/>
+      <c r="D273" s="31" t="n"/>
+      <c r="E273" s="31" t="n"/>
+      <c r="F273" s="31" t="n"/>
+    </row>
+    <row r="274" ht="24" customHeight="1">
+      <c r="A274" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B274" s="30" t="inlineStr">
+        <is>
+          <t>Admins get a monthly rollup focus, so it's low-pressure.</t>
+        </is>
+      </c>
+      <c r="C274" s="31" t="n"/>
+      <c r="D274" s="31" t="n"/>
+      <c r="E274" s="31" t="n"/>
+      <c r="F274" s="31" t="n"/>
+    </row>
+    <row r="275" ht="26" customHeight="1">
+      <c r="A275" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ Good to know · Coaching text is for a teacher's personal growth. We recommend using it as a support tool, not for evaluation/discipline.</t>
+        </is>
+      </c>
+      <c r="B275" s="35" t="n"/>
+      <c r="C275" s="35" t="n"/>
+      <c r="D275" s="35" t="n"/>
+      <c r="E275" s="35" t="n"/>
+      <c r="F275" s="35" t="n"/>
+    </row>
+    <row r="276" ht="30" customHeight="1">
+      <c r="A276" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · For teachers whose quality score stays low, coach them together with the teacher training manual.</t>
+        </is>
+      </c>
+      <c r="B276" s="33" t="n"/>
+      <c r="C276" s="33" t="n"/>
+      <c r="D276" s="33" t="n"/>
+      <c r="E276" s="33" t="n"/>
+      <c r="F276" s="33" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="208">
+  <mergeCells count="251">
     <mergeCell ref="B106:F106"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B194:F194"/>
+    <mergeCell ref="B252:F252"/>
     <mergeCell ref="B90:F90"/>
     <mergeCell ref="A189:F189"/>
+    <mergeCell ref="B261:F261"/>
     <mergeCell ref="A158:F158"/>
     <mergeCell ref="B122:F122"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="B131:F131"/>
+    <mergeCell ref="B236:F236"/>
     <mergeCell ref="B214:F214"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B180:F180"/>
     <mergeCell ref="B223:F223"/>
+    <mergeCell ref="B238:F238"/>
     <mergeCell ref="B195:F195"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B253:F253"/>
     <mergeCell ref="A159:F159"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="A200:F200"/>
+    <mergeCell ref="B250:F250"/>
     <mergeCell ref="A81:F81"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="B53:F53"/>
+    <mergeCell ref="A265:F265"/>
+    <mergeCell ref="B234:F234"/>
     <mergeCell ref="B172:F172"/>
     <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B270:F270"/>
     <mergeCell ref="B174:F174"/>
     <mergeCell ref="B108:F108"/>
     <mergeCell ref="B186:F186"/>
+    <mergeCell ref="A258:F258"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="B118:F118"/>
     <mergeCell ref="B143:F143"/>
+    <mergeCell ref="A257:F257"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A60:F60"/>
@@ -4428,15 +5075,18 @@
     <mergeCell ref="B142:F142"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="B213:F213"/>
+    <mergeCell ref="A241:F241"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="A124:F124"/>
     <mergeCell ref="B144:F144"/>
+    <mergeCell ref="B233:F233"/>
     <mergeCell ref="B227:F227"/>
     <mergeCell ref="B224:F224"/>
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B185:F185"/>
     <mergeCell ref="B134:F134"/>
+    <mergeCell ref="A267:F267"/>
     <mergeCell ref="A149:F149"/>
     <mergeCell ref="B121:F121"/>
     <mergeCell ref="A101:F101"/>
@@ -4448,6 +5098,7 @@
     <mergeCell ref="B111:F111"/>
     <mergeCell ref="B120:F120"/>
     <mergeCell ref="B98:F98"/>
+    <mergeCell ref="A254:F254"/>
     <mergeCell ref="A135:F135"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B8:F8"/>
@@ -4465,24 +5116,30 @@
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A176:F176"/>
+    <mergeCell ref="A232:F232"/>
     <mergeCell ref="A114:F114"/>
+    <mergeCell ref="B269:F269"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="B74:F74"/>
+    <mergeCell ref="B239:F239"/>
     <mergeCell ref="B153:F153"/>
     <mergeCell ref="A169:F169"/>
     <mergeCell ref="A178:F178"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B251:F251"/>
     <mergeCell ref="B76:F76"/>
     <mergeCell ref="B204:F204"/>
     <mergeCell ref="B216:F216"/>
     <mergeCell ref="B85:F85"/>
     <mergeCell ref="B173:F173"/>
+    <mergeCell ref="B271:F271"/>
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="A137:F137"/>
     <mergeCell ref="B109:F109"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B62:F62"/>
+    <mergeCell ref="A268:F268"/>
     <mergeCell ref="A217:F217"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B193:F193"/>
@@ -4491,19 +5148,28 @@
     <mergeCell ref="B202:F202"/>
     <mergeCell ref="A145:F145"/>
     <mergeCell ref="B215:F215"/>
+    <mergeCell ref="B273:F273"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A210:F210"/>
     <mergeCell ref="A179:F179"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A242:F242"/>
+    <mergeCell ref="B263:F263"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B152:F152"/>
+    <mergeCell ref="B272:F272"/>
     <mergeCell ref="B161:F161"/>
     <mergeCell ref="A116:F116"/>
+    <mergeCell ref="B259:F259"/>
+    <mergeCell ref="A244:F244"/>
     <mergeCell ref="B181:F181"/>
     <mergeCell ref="B225:F225"/>
+    <mergeCell ref="A231:F231"/>
+    <mergeCell ref="B274:F274"/>
     <mergeCell ref="B191:F191"/>
     <mergeCell ref="B73:F73"/>
+    <mergeCell ref="B249:F249"/>
     <mergeCell ref="B87:F87"/>
     <mergeCell ref="A93:F93"/>
     <mergeCell ref="A68:F68"/>
@@ -4512,6 +5178,9 @@
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A83:F83"/>
     <mergeCell ref="B226:F226"/>
+    <mergeCell ref="A245:F245"/>
+    <mergeCell ref="A276:F276"/>
+    <mergeCell ref="B260:F260"/>
     <mergeCell ref="A166:F166"/>
     <mergeCell ref="B183:F183"/>
     <mergeCell ref="B65:F65"/>
@@ -4540,6 +5209,7 @@
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="A128:F128"/>
     <mergeCell ref="B100:F100"/>
+    <mergeCell ref="A255:F255"/>
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="B165:F165"/>
@@ -4548,16 +5218,22 @@
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B155:F155"/>
+    <mergeCell ref="B264:F264"/>
     <mergeCell ref="A104:F104"/>
+    <mergeCell ref="B247:F247"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A113:F113"/>
     <mergeCell ref="B130:F130"/>
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="B248:F248"/>
+    <mergeCell ref="B262:F262"/>
     <mergeCell ref="A219:F219"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="B151:F151"/>
+    <mergeCell ref="B235:F235"/>
+    <mergeCell ref="B240:F240"/>
     <mergeCell ref="B67:F67"/>
     <mergeCell ref="B61:F61"/>
     <mergeCell ref="A4:F4"/>
@@ -4574,9 +5250,11 @@
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="A220:F220"/>
+    <mergeCell ref="B246:F246"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="A148:F148"/>
     <mergeCell ref="B211:F211"/>
+    <mergeCell ref="A275:F275"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B95:F95"/>
@@ -4592,6 +5270,7 @@
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B97:F97"/>
     <mergeCell ref="A25:F25"/>
+    <mergeCell ref="B237:F237"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
deploy: 2026-07-14 19:27 (build 20260714192715)
</commit_message>
<xml_diff>
--- a/cloudflare-deploy/public/library/admin/admin-en.xlsx
+++ b/cloudflare-deploy/public/library/admin/admin-en.xlsx
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1943,6 +1943,141 @@
       <c r="E28" s="15" t="inlineStr">
         <is>
           <t>For teachers whose quality score stays low, coach them together with the teacher training manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>📱</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>QR Attendance Check-in</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Open the QR Attendance card in the admin menu and generate your academy's QR code. → Print the QR and post it at the entrance or front desk. → Students scan with their phone camera and check in on the check-in screen. → Watch today's arrivals and times live on the dashboard's attendance view.</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>Stand a tablet at the desk during arrival hours so students can scan without queuing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>📞</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Consultation Booking Management</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Open the Consultation Booking card in the admin menu. → Register a new booking (name, contact, preferred time) or review incoming ones. → After the consult, set the status to done and leave a note. → Carry it forward: consult → level test → enrollment.</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>A quick follow-up call the day after a consult noticeably lifts enrollment conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>🎁</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Friend-Referral Rewards</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Open the Referral Rewards card in the admin menu. → Review the list of referrer · referred friend · enrollment status. → For qualifying cases, process the reward payout (points, gift vouchers, etc.).</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>Pair it with a 'refer a friend' event before each semester and watch inquiries jump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>🗓️</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Approving Postpone/Change Requests</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Open the Class Postpone/Change Requests card in the admin menu. → Review each pending request's teacher · class · reason. → Press Approve or Decline — the result flows to the schedule and the teacher.</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>Clearing pending requests every morning prevents same-day confusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>💬</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>Share Library Links via KakaoTalk</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>In the admin Library, press 💬 Copy KakaoTalk link next to the file. → Paste it into the KakaoTalk chat room. → Recipients tap the link to watch or download in original quality.</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="inlineStr">
+        <is>
+          <t>In a parents' group chat, one video-guide link does all the explaining.</t>
         </is>
       </c>
     </row>
@@ -1960,7 +2095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5018,8 +5153,602 @@
       <c r="E276" s="33" t="n"/>
       <c r="F276" s="33" t="n"/>
     </row>
+    <row r="278" ht="26" customHeight="1">
+      <c r="A278" s="21" t="inlineStr">
+        <is>
+          <t>26  📱 QR Attendance Check-in  —  One scan and attendance is done</t>
+        </is>
+      </c>
+      <c r="B278" s="22" t="n"/>
+      <c r="C278" s="22" t="n"/>
+      <c r="D278" s="22" t="n"/>
+      <c r="E278" s="22" t="n"/>
+      <c r="F278" s="22" t="n"/>
+    </row>
+    <row r="279" ht="42" customHeight="1">
+      <c r="A279" s="23" t="inlineStr">
+        <is>
+          <t>📖 Post an attendance QR code at the entrance, and the moment a student scans it with their phone, attendance is recorded automatically. The admin dashboard shows today's attendance in real time — no more paper rosters.</t>
+        </is>
+      </c>
+      <c r="B279" s="24" t="n"/>
+      <c r="C279" s="24" t="n"/>
+      <c r="D279" s="24" t="n"/>
+      <c r="E279" s="24" t="n"/>
+      <c r="F279" s="24" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B280" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="30" customHeight="1">
+      <c r="A281" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B281" s="28" t="inlineStr">
+        <is>
+          <t>Open the QR Attendance card in the admin menu and generate your academy's QR code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="30" customHeight="1">
+      <c r="A282" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B282" s="28" t="inlineStr">
+        <is>
+          <t>Print the QR and post it at the entrance or front desk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="30" customHeight="1">
+      <c r="A283" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B283" s="28" t="inlineStr">
+        <is>
+          <t>Students scan with their phone camera and check in on the check-in screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="30" customHeight="1">
+      <c r="A284" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B284" s="28" t="inlineStr">
+        <is>
+          <t>Watch today's arrivals and times live on the dashboard's attendance view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="24" customHeight="1">
+      <c r="A285" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B285" s="30" t="inlineStr">
+        <is>
+          <t>Arrival times are recorded automatically — fast and accurate.</t>
+        </is>
+      </c>
+      <c r="C285" s="31" t="n"/>
+      <c r="D285" s="31" t="n"/>
+      <c r="E285" s="31" t="n"/>
+      <c r="F285" s="31" t="n"/>
+    </row>
+    <row r="286" ht="24" customHeight="1">
+      <c r="A286" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B286" s="30" t="inlineStr">
+        <is>
+          <t>Attendance data flows into student management and reports.</t>
+        </is>
+      </c>
+      <c r="C286" s="31" t="n"/>
+      <c r="D286" s="31" t="n"/>
+      <c r="E286" s="31" t="n"/>
+      <c r="F286" s="31" t="n"/>
+    </row>
+    <row r="287" ht="26" customHeight="1">
+      <c r="A287" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ Good to know · The QR code is unique to your academy. Keep it from being shared outside.</t>
+        </is>
+      </c>
+      <c r="B287" s="35" t="n"/>
+      <c r="C287" s="35" t="n"/>
+      <c r="D287" s="35" t="n"/>
+      <c r="E287" s="35" t="n"/>
+      <c r="F287" s="35" t="n"/>
+    </row>
+    <row r="288" ht="30" customHeight="1">
+      <c r="A288" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · Stand a tablet at the desk during arrival hours so students can scan without queuing.</t>
+        </is>
+      </c>
+      <c r="B288" s="33" t="n"/>
+      <c r="C288" s="33" t="n"/>
+      <c r="D288" s="33" t="n"/>
+      <c r="E288" s="33" t="n"/>
+      <c r="F288" s="33" t="n"/>
+    </row>
+    <row r="290" ht="26" customHeight="1">
+      <c r="A290" s="21" t="inlineStr">
+        <is>
+          <t>27  📞 Consultation Booking Management  —  From new inquiries to scheduled consults</t>
+        </is>
+      </c>
+      <c r="B290" s="22" t="n"/>
+      <c r="C290" s="22" t="n"/>
+      <c r="D290" s="22" t="n"/>
+      <c r="E290" s="22" t="n"/>
+      <c r="F290" s="22" t="n"/>
+    </row>
+    <row r="291" ht="42" customHeight="1">
+      <c r="A291" s="23" t="inlineStr">
+        <is>
+          <t>📖 Take consultation bookings from parents and prospects and manage them on one screen. Track each booking's schedule and status (pending/done) and carry the consult onward toward enrollment.</t>
+        </is>
+      </c>
+      <c r="B291" s="24" t="n"/>
+      <c r="C291" s="24" t="n"/>
+      <c r="D291" s="24" t="n"/>
+      <c r="E291" s="24" t="n"/>
+      <c r="F291" s="24" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B292" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="30" customHeight="1">
+      <c r="A293" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B293" s="28" t="inlineStr">
+        <is>
+          <t>Open the Consultation Booking card in the admin menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="30" customHeight="1">
+      <c r="A294" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B294" s="28" t="inlineStr">
+        <is>
+          <t>Register a new booking (name, contact, preferred time) or review incoming ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="30" customHeight="1">
+      <c r="A295" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B295" s="28" t="inlineStr">
+        <is>
+          <t>After the consult, set the status to done and leave a note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="30" customHeight="1">
+      <c r="A296" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B296" s="28" t="inlineStr">
+        <is>
+          <t>Carry it forward: consult → level test → enrollment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="24" customHeight="1">
+      <c r="A297" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B297" s="30" t="inlineStr">
+        <is>
+          <t>Bookings live in one place, so no consult slips through.</t>
+        </is>
+      </c>
+      <c r="C297" s="31" t="n"/>
+      <c r="D297" s="31" t="n"/>
+      <c r="E297" s="31" t="n"/>
+      <c r="F297" s="31" t="n"/>
+    </row>
+    <row r="298" ht="24" customHeight="1">
+      <c r="A298" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B298" s="30" t="inlineStr">
+        <is>
+          <t>Consult history makes repeat inquiries easy to handle.</t>
+        </is>
+      </c>
+      <c r="C298" s="31" t="n"/>
+      <c r="D298" s="31" t="n"/>
+      <c r="E298" s="31" t="n"/>
+      <c r="F298" s="31" t="n"/>
+    </row>
+    <row r="299" ht="30" customHeight="1">
+      <c r="A299" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · A quick follow-up call the day after a consult noticeably lifts enrollment conversion.</t>
+        </is>
+      </c>
+      <c r="B299" s="33" t="n"/>
+      <c r="C299" s="33" t="n"/>
+      <c r="D299" s="33" t="n"/>
+      <c r="E299" s="33" t="n"/>
+      <c r="F299" s="33" t="n"/>
+    </row>
+    <row r="301" ht="26" customHeight="1">
+      <c r="A301" s="21" t="inlineStr">
+        <is>
+          <t>28  🎁 Friend-Referral Rewards  —  Track referrals · pay out rewards</t>
+        </is>
+      </c>
+      <c r="B301" s="22" t="n"/>
+      <c r="C301" s="22" t="n"/>
+      <c r="D301" s="22" t="n"/>
+      <c r="E301" s="22" t="n"/>
+      <c r="F301" s="22" t="n"/>
+    </row>
+    <row r="302" ht="42" customHeight="1">
+      <c r="A302" s="23" t="inlineStr">
+        <is>
+          <t>📖 See the referral status of enrolled students bringing friends, and process reward payouts. Who referred whom, and whether the reward was paid — all on one screen, turning word-of-mouth into a system.</t>
+        </is>
+      </c>
+      <c r="B302" s="24" t="n"/>
+      <c r="C302" s="24" t="n"/>
+      <c r="D302" s="24" t="n"/>
+      <c r="E302" s="24" t="n"/>
+      <c r="F302" s="24" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B303" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="30" customHeight="1">
+      <c r="A304" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B304" s="28" t="inlineStr">
+        <is>
+          <t>Open the Referral Rewards card in the admin menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="30" customHeight="1">
+      <c r="A305" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B305" s="28" t="inlineStr">
+        <is>
+          <t>Review the list of referrer · referred friend · enrollment status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="30" customHeight="1">
+      <c r="A306" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B306" s="28" t="inlineStr">
+        <is>
+          <t>For qualifying cases, process the reward payout (points, gift vouchers, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="24" customHeight="1">
+      <c r="A307" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B307" s="30" t="inlineStr">
+        <is>
+          <t>Referral history is kept as data — transparent, no disputes.</t>
+        </is>
+      </c>
+      <c r="C307" s="31" t="n"/>
+      <c r="D307" s="31" t="n"/>
+      <c r="E307" s="31" t="n"/>
+      <c r="F307" s="31" t="n"/>
+    </row>
+    <row r="308" ht="24" customHeight="1">
+      <c r="A308" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B308" s="30" t="inlineStr">
+        <is>
+          <t>Linking rewards to student points and the shop multiplies the effect.</t>
+        </is>
+      </c>
+      <c r="C308" s="31" t="n"/>
+      <c r="D308" s="31" t="n"/>
+      <c r="E308" s="31" t="n"/>
+      <c r="F308" s="31" t="n"/>
+    </row>
+    <row r="309" ht="30" customHeight="1">
+      <c r="A309" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · Pair it with a 'refer a friend' event before each semester and watch inquiries jump.</t>
+        </is>
+      </c>
+      <c r="B309" s="33" t="n"/>
+      <c r="C309" s="33" t="n"/>
+      <c r="D309" s="33" t="n"/>
+      <c r="E309" s="33" t="n"/>
+      <c r="F309" s="33" t="n"/>
+    </row>
+    <row r="311" ht="26" customHeight="1">
+      <c r="A311" s="21" t="inlineStr">
+        <is>
+          <t>29  🗓️ Approving Postpone/Change Requests  —  Review and approve teacher-submitted requests</t>
+        </is>
+      </c>
+      <c r="B311" s="22" t="n"/>
+      <c r="C311" s="22" t="n"/>
+      <c r="D311" s="22" t="n"/>
+      <c r="E311" s="22" t="n"/>
+      <c r="F311" s="22" t="n"/>
+    </row>
+    <row r="312" ht="42" customHeight="1">
+      <c r="A312" s="23" t="inlineStr">
+        <is>
+          <t>📖 Class postpone and time-change requests submitted by teachers gather on the admin screen in real time. Check the reason and approve or decline — the schedule updates immediately, replacing phone-and-messenger juggling with one screen.</t>
+        </is>
+      </c>
+      <c r="B312" s="24" t="n"/>
+      <c r="C312" s="24" t="n"/>
+      <c r="D312" s="24" t="n"/>
+      <c r="E312" s="24" t="n"/>
+      <c r="F312" s="24" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B313" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="30" customHeight="1">
+      <c r="A314" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B314" s="28" t="inlineStr">
+        <is>
+          <t>Open the Class Postpone/Change Requests card in the admin menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="30" customHeight="1">
+      <c r="A315" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B315" s="28" t="inlineStr">
+        <is>
+          <t>Review each pending request's teacher · class · reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="30" customHeight="1">
+      <c r="A316" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B316" s="28" t="inlineStr">
+        <is>
+          <t>Press Approve or Decline — the result flows to the schedule and the teacher.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="24" customHeight="1">
+      <c r="A317" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B317" s="30" t="inlineStr">
+        <is>
+          <t>Request and decision history is kept, so everything stays transparent.</t>
+        </is>
+      </c>
+      <c r="C317" s="31" t="n"/>
+      <c r="D317" s="31" t="n"/>
+      <c r="E317" s="31" t="n"/>
+      <c r="F317" s="31" t="n"/>
+    </row>
+    <row r="318" ht="24" customHeight="1">
+      <c r="A318" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B318" s="30" t="inlineStr">
+        <is>
+          <t>For changes parents should know about, follow approval with a notification.</t>
+        </is>
+      </c>
+      <c r="C318" s="31" t="n"/>
+      <c r="D318" s="31" t="n"/>
+      <c r="E318" s="31" t="n"/>
+      <c r="F318" s="31" t="n"/>
+    </row>
+    <row r="319" ht="30" customHeight="1">
+      <c r="A319" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · Clearing pending requests every morning prevents same-day confusion.</t>
+        </is>
+      </c>
+      <c r="B319" s="33" t="n"/>
+      <c r="C319" s="33" t="n"/>
+      <c r="D319" s="33" t="n"/>
+      <c r="E319" s="33" t="n"/>
+      <c r="F319" s="33" t="n"/>
+    </row>
+    <row r="321" ht="26" customHeight="1">
+      <c r="A321" s="21" t="inlineStr">
+        <is>
+          <t>30  💬 Share Library Links via KakaoTalk  —  Send videos &amp; docs in original quality</t>
+        </is>
+      </c>
+      <c r="B321" s="22" t="n"/>
+      <c r="C321" s="22" t="n"/>
+      <c r="D321" s="22" t="n"/>
+      <c r="E321" s="22" t="n"/>
+      <c r="F321" s="22" t="n"/>
+    </row>
+    <row r="322" ht="42" customHeight="1">
+      <c r="A322" s="23" t="inlineStr">
+        <is>
+          <t>📖 Every guide and video in the library now has a '💬 Copy KakaoTalk link' button. Attaching a file to KakaoTalk crushes the quality, but sending a link plays the original as-is. One tap copies the link — guiding parents and teachers gets much easier.</t>
+        </is>
+      </c>
+      <c r="B322" s="24" t="n"/>
+      <c r="C322" s="24" t="n"/>
+      <c r="D322" s="24" t="n"/>
+      <c r="E322" s="24" t="n"/>
+      <c r="F322" s="24" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="25" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B323" s="26" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="30" customHeight="1">
+      <c r="A324" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B324" s="28" t="inlineStr">
+        <is>
+          <t>In the admin Library, press 💬 Copy KakaoTalk link next to the file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="30" customHeight="1">
+      <c r="A325" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B325" s="28" t="inlineStr">
+        <is>
+          <t>Paste it into the KakaoTalk chat room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="30" customHeight="1">
+      <c r="A326" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B326" s="28" t="inlineStr">
+        <is>
+          <t>Recipients tap the link to watch or download in original quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="24" customHeight="1">
+      <c r="A327" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B327" s="30" t="inlineStr">
+        <is>
+          <t>For videos, link sharing = original quality; file attachments degrade it.</t>
+        </is>
+      </c>
+      <c r="C327" s="31" t="n"/>
+      <c r="D327" s="31" t="n"/>
+      <c r="E327" s="31" t="n"/>
+      <c r="F327" s="31" t="n"/>
+    </row>
+    <row r="328" ht="24" customHeight="1">
+      <c r="A328" s="29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="B328" s="30" t="inlineStr">
+        <is>
+          <t>Works the same for PDFs, PPTs, and videos anywhere in the library.</t>
+        </is>
+      </c>
+      <c r="C328" s="31" t="n"/>
+      <c r="D328" s="31" t="n"/>
+      <c r="E328" s="31" t="n"/>
+      <c r="F328" s="31" t="n"/>
+    </row>
+    <row r="329" ht="26" customHeight="1">
+      <c r="A329" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ Good to know · Anyone with the link can open it. For internal-only material, check who you share with.</t>
+        </is>
+      </c>
+      <c r="B329" s="35" t="n"/>
+      <c r="C329" s="35" t="n"/>
+      <c r="D329" s="35" t="n"/>
+      <c r="E329" s="35" t="n"/>
+      <c r="F329" s="35" t="n"/>
+    </row>
+    <row r="330" ht="30" customHeight="1">
+      <c r="A330" s="32" t="inlineStr">
+        <is>
+          <t>💡 Tip · In a parents' group chat, one video-guide link does all the explaining.</t>
+        </is>
+      </c>
+      <c r="B330" s="33" t="n"/>
+      <c r="C330" s="33" t="n"/>
+      <c r="D330" s="33" t="n"/>
+      <c r="E330" s="33" t="n"/>
+      <c r="F330" s="33" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="251">
+  <mergeCells count="300">
     <mergeCell ref="B106:F106"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
@@ -5031,6 +5760,7 @@
     <mergeCell ref="A189:F189"/>
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="A158:F158"/>
+    <mergeCell ref="B292:F292"/>
     <mergeCell ref="B122:F122"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="A3:F3"/>
@@ -5039,23 +5769,31 @@
     <mergeCell ref="B214:F214"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B27:F27"/>
+    <mergeCell ref="A301:F301"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B180:F180"/>
     <mergeCell ref="B223:F223"/>
     <mergeCell ref="B238:F238"/>
+    <mergeCell ref="B294:F294"/>
+    <mergeCell ref="B307:F307"/>
+    <mergeCell ref="B303:F303"/>
     <mergeCell ref="B195:F195"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="B253:F253"/>
+    <mergeCell ref="A321:F321"/>
     <mergeCell ref="A159:F159"/>
+    <mergeCell ref="A290:F290"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="A200:F200"/>
     <mergeCell ref="B250:F250"/>
+    <mergeCell ref="B328:F328"/>
     <mergeCell ref="A81:F81"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="A265:F265"/>
     <mergeCell ref="B234:F234"/>
+    <mergeCell ref="A288:F288"/>
     <mergeCell ref="B172:F172"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B270:F270"/>
@@ -5063,21 +5801,27 @@
     <mergeCell ref="B108:F108"/>
     <mergeCell ref="B186:F186"/>
     <mergeCell ref="A258:F258"/>
+    <mergeCell ref="A329:F329"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="B118:F118"/>
     <mergeCell ref="B143:F143"/>
     <mergeCell ref="A257:F257"/>
     <mergeCell ref="B30:F30"/>
+    <mergeCell ref="A291:F291"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A60:F60"/>
+    <mergeCell ref="B281:F281"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B142:F142"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="B213:F213"/>
     <mergeCell ref="A241:F241"/>
+    <mergeCell ref="B313:F313"/>
     <mergeCell ref="B160:F160"/>
+    <mergeCell ref="B305:F305"/>
     <mergeCell ref="A124:F124"/>
+    <mergeCell ref="B306:F306"/>
     <mergeCell ref="B144:F144"/>
     <mergeCell ref="B233:F233"/>
     <mergeCell ref="B227:F227"/>
@@ -5095,13 +5839,17 @@
     <mergeCell ref="B105:F105"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B228:F228"/>
+    <mergeCell ref="A278:F278"/>
     <mergeCell ref="B111:F111"/>
+    <mergeCell ref="B293:F293"/>
     <mergeCell ref="B120:F120"/>
     <mergeCell ref="B98:F98"/>
     <mergeCell ref="A254:F254"/>
+    <mergeCell ref="A311:F311"/>
     <mergeCell ref="A135:F135"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B318:F318"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B175:F175"/>
     <mergeCell ref="B88:F88"/>
@@ -5111,7 +5859,9 @@
     <mergeCell ref="A199:F199"/>
     <mergeCell ref="B171:F171"/>
     <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B308:F308"/>
     <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B317:F317"/>
     <mergeCell ref="A127:F127"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="A48:F48"/>
@@ -5122,7 +5872,9 @@
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="B74:F74"/>
+    <mergeCell ref="B304:F304"/>
     <mergeCell ref="B239:F239"/>
+    <mergeCell ref="A319:F319"/>
     <mergeCell ref="B153:F153"/>
     <mergeCell ref="A169:F169"/>
     <mergeCell ref="A178:F178"/>
@@ -5132,15 +5884,18 @@
     <mergeCell ref="B204:F204"/>
     <mergeCell ref="B216:F216"/>
     <mergeCell ref="B85:F85"/>
+    <mergeCell ref="B296:F296"/>
     <mergeCell ref="B173:F173"/>
     <mergeCell ref="B271:F271"/>
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="A137:F137"/>
     <mergeCell ref="B109:F109"/>
     <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B280:F280"/>
     <mergeCell ref="B62:F62"/>
     <mergeCell ref="A268:F268"/>
     <mergeCell ref="A217:F217"/>
+    <mergeCell ref="A330:F330"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B193:F193"/>
     <mergeCell ref="B150:F150"/>
@@ -5150,8 +5905,11 @@
     <mergeCell ref="B215:F215"/>
     <mergeCell ref="B273:F273"/>
     <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B282:F282"/>
     <mergeCell ref="A210:F210"/>
+    <mergeCell ref="B295:F295"/>
     <mergeCell ref="A179:F179"/>
+    <mergeCell ref="B325:F325"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="A71:F71"/>
     <mergeCell ref="A242:F242"/>
@@ -5159,9 +5917,12 @@
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B152:F152"/>
     <mergeCell ref="B272:F272"/>
+    <mergeCell ref="A322:F322"/>
     <mergeCell ref="B161:F161"/>
+    <mergeCell ref="B323:F323"/>
     <mergeCell ref="A116:F116"/>
     <mergeCell ref="B259:F259"/>
+    <mergeCell ref="A309:F309"/>
     <mergeCell ref="A244:F244"/>
     <mergeCell ref="B181:F181"/>
     <mergeCell ref="B225:F225"/>
@@ -5170,6 +5931,7 @@
     <mergeCell ref="B191:F191"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B249:F249"/>
+    <mergeCell ref="A299:F299"/>
     <mergeCell ref="B87:F87"/>
     <mergeCell ref="A93:F93"/>
     <mergeCell ref="A68:F68"/>
@@ -5182,10 +5944,12 @@
     <mergeCell ref="A276:F276"/>
     <mergeCell ref="B260:F260"/>
     <mergeCell ref="A166:F166"/>
+    <mergeCell ref="A279:F279"/>
     <mergeCell ref="B183:F183"/>
     <mergeCell ref="B65:F65"/>
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="B192:F192"/>
+    <mergeCell ref="B324:F324"/>
     <mergeCell ref="B201:F201"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="B139:F139"/>
@@ -5197,7 +5961,9 @@
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="A168:F168"/>
+    <mergeCell ref="B284:F284"/>
     <mergeCell ref="B63:F63"/>
+    <mergeCell ref="A287:F287"/>
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="B212:F212"/>
@@ -5207,8 +5973,10 @@
     <mergeCell ref="B110:F110"/>
     <mergeCell ref="B203:F203"/>
     <mergeCell ref="B221:F221"/>
+    <mergeCell ref="B286:F286"/>
     <mergeCell ref="A128:F128"/>
     <mergeCell ref="B100:F100"/>
+    <mergeCell ref="B327:F327"/>
     <mergeCell ref="A255:F255"/>
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="A37:F37"/>
@@ -5219,12 +5987,14 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B155:F155"/>
     <mergeCell ref="B264:F264"/>
+    <mergeCell ref="B326:F326"/>
     <mergeCell ref="A104:F104"/>
     <mergeCell ref="B247:F247"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A113:F113"/>
     <mergeCell ref="B130:F130"/>
     <mergeCell ref="B77:F77"/>
+    <mergeCell ref="A302:F302"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="B248:F248"/>
@@ -5235,6 +6005,8 @@
     <mergeCell ref="B235:F235"/>
     <mergeCell ref="B240:F240"/>
     <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B297:F297"/>
+    <mergeCell ref="A312:F312"/>
     <mergeCell ref="B61:F61"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B132:F132"/>
@@ -5249,12 +6021,17 @@
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B205:F205"/>
+    <mergeCell ref="B283:F283"/>
+    <mergeCell ref="B314:F314"/>
     <mergeCell ref="A220:F220"/>
     <mergeCell ref="B246:F246"/>
+    <mergeCell ref="B298:F298"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="A148:F148"/>
     <mergeCell ref="B211:F211"/>
     <mergeCell ref="A275:F275"/>
+    <mergeCell ref="B285:F285"/>
+    <mergeCell ref="B316:F316"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B95:F95"/>
@@ -5264,6 +6041,7 @@
     <mergeCell ref="A197:F197"/>
     <mergeCell ref="B51:F51"/>
     <mergeCell ref="A146:F146"/>
+    <mergeCell ref="B315:F315"/>
     <mergeCell ref="B79:F79"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="A187:F187"/>

</xml_diff>